<commit_message>
Add provider-neutral catalog evidence layer
</commit_message>
<xml_diff>
--- a/artifacts/AI_Build_Crew_Agentic_AI_PRD.xlsx
+++ b/artifacts/AI_Build_Crew_Agentic_AI_PRD.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1700eec859a14048"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4088bf59256349e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1037,7 +1037,7 @@
         <x:v>What single end-to-end loop will the prototype prove?</x:v>
       </x:c>
       <x:c r="F30" s="37" t="str">
-        <x:v>Enter one AI workload plan → identify missing constraints → compare a limited model catalog → calculate low/expected/high cost → filter and rank candidates → explain the recommendation and tuning options → let the human approve or override → display a saved decision brief.</x:v>
+        <x:v>Enter one AI workload plan → identify missing constraints → compare sourced catalog facts across OpenAI, Google, and Anthropic → calculate low/expected/high cost → rank only candidates with shared evidence → explain the recommendation and tuning options → let the human approve or override → display a saved decision brief.</x:v>
       </x:c>
       <x:c r="G30" s="37" t="str"/>
     </x:row>
@@ -1075,7 +1075,7 @@
         <x:v>List the fake data files, sample records, policies, or examples used in the prototype.</x:v>
       </x:c>
       <x:c r="F32" s="23" t="str">
-        <x:v>Planned demo-safe inputs: models.json with a limited timestamped sample catalog; workload_cases.json with at least eight fictional plans; eligibility_rules.json; risk_policy.md; cost_scenarios.json; recommendation_expected_results.json; and a fictional RAG customer-support workload used in the demo. Public prices may replace sample prices only after source and freshness checks are implemented.</x:v>
+        <x:v>Implemented demo-safe inputs: a versioned catalog containing dated published facts for three OpenAI, two Google Gemini, and three Anthropic Claude models; versioned intake, eligibility, and governance rules; deterministic cost scenarios; ten fictional evaluation cases; and a synthetic RAG customer-support workload used in the demo. No secret, customer, employer, medical, or proprietary data is required.</x:v>
       </x:c>
       <x:c r="G32" s="26" t="str"/>
     </x:row>
@@ -1151,7 +1151,7 @@
         <x:v>What does the prototype not do yet? Be honest and specific.</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>The alpha will cover a limited model catalog and a constrained set of task types. It will not prove universal model quality, purchase or provision access, automatically route production traffic, ingest secrets or protected data, monitor real production spend, approve regulated deployments, cover every provider fee, guarantee future pricing, or implement monetization and stored-value credits. Recommendations are planning support, not deployment authorization.</x:v>
+        <x:v>The alpha compares sourced catalog facts across three providers, but only the evaluated baseline can enter the recommendation ranking. It will not infer universal model quality, purchase or provision access, automatically route production traffic, ingest secrets or protected data, monitor real production spend, approve regulated deployments, cover every provider fee, guarantee future pricing, or implement monetization and stored-value credits. The tool is authoritative for its versioned inputs, sourced facts, deterministic calculations, and recorded policy disposition; CT remains the decision owner.</x:v>
       </x:c>
       <x:c r="G36" s="26" t="str"/>
     </x:row>
@@ -1286,7 +1286,7 @@
         <x:v>What is the smallest safe launch or pilot path?</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>Begin with CT and synthetic workloads using the limited OpenAI catalog. Run three real non-sensitive planning sessions plus high-risk, stale-catalog, and unsupported-modality failure demos. Next invite three to five product builders with fictional or sanitized plans. Add Google Gemini and Anthropic Claude only through the normalized, versioned catalog after source, freshness, capability, and ranking-bias tests pass.</x:v>
+        <x:v>Begin with CT and synthetic or non-sensitive workloads using the three-provider catalog. Run three real planning sessions plus high-risk, stale-catalog, and unsupported-modality failure demos. Next invite three to five product builders with fictional or sanitized plans. Connect Google Gemini and Anthropic Claude to shared live evaluation only after provider-key, budget, synthetic-case, adapter, source, freshness, and ranking-bias tests pass.</x:v>
       </x:c>
       <x:c r="G43" s="26" t="str"/>
     </x:row>
@@ -1305,7 +1305,7 @@
         <x:v>How will your video cover intro, problem, discovery, solution demo, eval rigor, impact, and launch plan?</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>0:00–0:25 Explain fragmented model choice and bad defaults. 0:25–0:45 Introduce AI Build Crew and CT. 0:45–1:15 Show prompt-first routing and Known/Assumed/Unknown. 1:15–1:45 Show scenarios, rule eligibility, recommendation, and alternative deltas. 1:45–2:10 Show independent Evaluation, Audit, Governance, and CT ownership. 2:10–2:30 State 10/10 evidence, limitations, and the Google/Anthropic next step.</x:v>
+        <x:v>0:00–0:25 Explain fragmented model choice and bad defaults. 0:25–0:45 Introduce AI Build Crew and CT. 0:45–1:15 Show prompt-first routing and Known/Assumed/Unknown. 1:15–1:45 Show three-provider catalog facts, scenarios, rule eligibility, and evidence-gated ranking. 1:45–2:10 Show independent Evaluation, Audit, Governance, and CT ownership. 2:10–2:30 State 10/10 evidence, limitations, and shared live evaluation as the next step.</x:v>
       </x:c>
       <x:c r="G44" s="26" t="str"/>
     </x:row>
@@ -1364,7 +1364,7 @@
         <x:v>Does the 2–3 minute video show the product clearly, concisely, and persuasively?</x:v>
       </x:c>
       <x:c r="F47" s="48" t="str">
-        <x:v>READY TO RECORD. A timed 2:30 script and operator checklist are complete. Before submission, record it, verify runtime, confirm the high-risk review state is visible, and check that the narration matches the PRD, evaluation, limitations, and provider-expansion plan.</x:v>
+        <x:v>READY TO RECORD. A timed 2:30 script and operator checklist are complete. Before submission, record it, verify runtime, confirm the high-risk review state is visible, and check that the narration matches the PRD, evaluation, limitations, three-provider catalog, and shared-evaluation next step.</x:v>
       </x:c>
       <x:c r="G47" s="27" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Productize governed alpha for first-time builders
</commit_message>
<xml_diff>
--- a/artifacts/AI_Build_Crew_Agentic_AI_PRD.xlsx
+++ b/artifacts/AI_Build_Crew_Agentic_AI_PRD.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4088bf59256349e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1c0b25e54fdd43b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -542,7 +542,7 @@
         <x:v>Your Name:</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>CT Tansted</x:v>
+        <x:v>BadLabz Product Team</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
@@ -568,7 +568,7 @@
         <x:v>Workflow / Project Choice:</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>A prompt-first planning workflow where a builder turns an incomplete AI idea into a transparent workload forecast, a deterministic rule-eligible model recommendation, independent evaluation/audit/governance evidence, and a final decision owned by CT.</x:v>
+        <x:v>A prompt-first planning workflow where a builder turns an incomplete AI idea into a transparent workload forecast, a deterministic rule-eligible model recommendation, independent evaluation/audit/governance evidence, and a final decision owned by the product builder.</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
       <x:c r="D5" s="1"/>
@@ -605,10 +605,10 @@
       <x:c r="B8" s="15" t="str">
         <x:v>Agentic AI PRD</x:v>
       </x:c>
-      <x:c r="C8" s="15" t="str"/>
-      <x:c r="D8" s="15" t="str"/>
-      <x:c r="E8" s="15" t="str"/>
-      <x:c r="F8" s="15" t="str"/>
+      <x:c r="C8" s="15"/>
+      <x:c r="D8" s="15"/>
+      <x:c r="E8" s="15"/>
+      <x:c r="F8" s="15"/>
       <x:c r="G8" s="15" t="str">
         <x:v>Faculty Feedback</x:v>
       </x:c>
@@ -653,12 +653,12 @@
         <x:v>Who is the specific user this agent helps?</x:v>
       </x:c>
       <x:c r="F10" s="31" t="str">
-        <x:v>The first user is CT, a product person and AI builder who must choose a suitable model, estimate likely operating cost, and explain the decision without a dedicated AI architect or AI FinOps specialist. The broader beachhead is product managers and small AI product teams planning multi-model workflows.</x:v>
-      </x:c>
-      <x:c r="G10" s="31" t="str"/>
+        <x:v>The first user is the product builder, a product person and AI builder who must choose a suitable model, estimate likely operating cost, and explain the decision without a dedicated AI architect or AI FinOps specialist. The broader beachhead is product managers and small AI product teams planning multi-model workflows.</x:v>
+      </x:c>
+      <x:c r="G10" s="31"/>
     </x:row>
     <x:row r="11" ht="88" customHeight="1">
-      <x:c r="A11" s="20" t="str"/>
+      <x:c r="A11" s="20"/>
       <x:c r="B11" s="20" t="str">
         <x:v>Project choice</x:v>
       </x:c>
@@ -674,10 +674,10 @@
       <x:c r="F11" s="23" t="str">
         <x:v>The recurring workflow is pre-build model selection and cost planning. The user turns a rough AI product idea into a workload description, researches candidate models and pricing, estimates token and workflow usage, compares cost/quality/latency/risk tradeoffs, identifies design optimizations, and prepares a decision for review.</x:v>
       </x:c>
-      <x:c r="G11" s="26" t="str"/>
+      <x:c r="G11" s="26"/>
     </x:row>
     <x:row r="12" ht="88" customHeight="1">
-      <x:c r="A12" s="20" t="str"/>
+      <x:c r="A12" s="20"/>
       <x:c r="B12" s="20" t="str">
         <x:v>Project choice</x:v>
       </x:c>
@@ -693,10 +693,10 @@
       <x:c r="F12" s="23" t="str">
         <x:v>The workflow starts when the user has an AI product idea, feature, agent, prompt workflow, or architecture decision and must choose a model and estimate cost before committing engineering effort or seeking approval.</x:v>
       </x:c>
-      <x:c r="G12" s="26" t="str"/>
+      <x:c r="G12" s="26"/>
     </x:row>
     <x:row r="13" ht="88" customHeight="1">
-      <x:c r="A13" s="20" t="str"/>
+      <x:c r="A13" s="20"/>
       <x:c r="B13" s="20" t="str">
         <x:v>Current state</x:v>
       </x:c>
@@ -712,10 +712,10 @@
       <x:c r="F13" s="23" t="str">
         <x:v>1. Describe the product idea informally. 2. Search provider pages and third-party comparisons. 3. Try to understand model capabilities and price units. 4. Guess input/output token volumes, number of calls, context, tools, retrieval, and loops. 5. Compare candidates manually, often in notes or a spreadsheet. 6. Select a familiar or premium model when evidence is unclear. 7. Revise the estimate when assumptions or prices change. 8. Explain the choice to reviewers without a consistent decision record.</x:v>
       </x:c>
-      <x:c r="G13" s="26" t="str"/>
+      <x:c r="G13" s="26"/>
     </x:row>
     <x:row r="14" ht="88" customHeight="1">
-      <x:c r="A14" s="20" t="str"/>
+      <x:c r="A14" s="20"/>
       <x:c r="B14" s="20" t="str">
         <x:v>Problem</x:v>
       </x:c>
@@ -731,10 +731,10 @@
       <x:c r="F14" s="23" t="str">
         <x:v>Information is fragmented and changes frequently. Prices use different categories, model names do not explain task fit, public benchmarks may not reflect the real workload, and builders often do not know how context, caching, tools, retrieval, or agent loops affect cost. This creates slow research, false precision, repeated work, defaulting to expensive models, and decisions that are difficult to defend.</x:v>
       </x:c>
-      <x:c r="G14" s="26" t="str"/>
+      <x:c r="G14" s="26"/>
     </x:row>
     <x:row r="15" ht="88" customHeight="1">
-      <x:c r="A15" s="20" t="str"/>
+      <x:c r="A15" s="20"/>
       <x:c r="B15" s="20" t="str">
         <x:v>Opportunity</x:v>
       </x:c>
@@ -750,10 +750,10 @@
       <x:c r="F15" s="23" t="str">
         <x:v>The agent should interview the user about intent and constraints, detect missing assumptions, retrieve a normalized model catalog, calculate scenarios, filter ineligible models, compare tradeoffs, recommend tuning, and produce a reviewable decision brief. An agent is a better fit than a static calculator because the required questions and recommendations change based on the workload, risk, missing information, and previous answers.</x:v>
       </x:c>
-      <x:c r="G15" s="26" t="str"/>
+      <x:c r="G15" s="26"/>
     </x:row>
     <x:row r="16" ht="88" customHeight="1">
-      <x:c r="A16" s="20" t="str"/>
+      <x:c r="A16" s="20"/>
       <x:c r="B16" s="20" t="str">
         <x:v>Data</x:v>
       </x:c>
@@ -769,10 +769,10 @@
       <x:c r="F16" s="23" t="str">
         <x:v>Create a synthetic model catalog with clearly marked sample prices and capabilities for development, plus at least eight fictional workload plans: customer-support classifier, document summarizer, code assistant, RAG Q&amp;A, image extraction, high-risk medical draft, agent with excessive loops, and a workload with missing data. Create policy rules for risk, required human review, stale pricing, missing capability evidence, and unsupported modalities. No customer, employer, medical, or proprietary data is required.</x:v>
       </x:c>
-      <x:c r="G16" s="26" t="str"/>
+      <x:c r="G16" s="26"/>
     </x:row>
     <x:row r="17" ht="88" customHeight="1">
-      <x:c r="A17" s="20" t="str"/>
+      <x:c r="A17" s="20"/>
       <x:c r="B17" s="20" t="str">
         <x:v>Safety</x:v>
       </x:c>
@@ -788,10 +788,10 @@
       <x:c r="F17" s="23" t="str">
         <x:v>The agent cannot claim a universally best model, invent price or capability facts, purchase or provision access, deploy a workload, approve a regulated or high-risk use case, or use protected data. A human must approve the final model decision, review any high-risk or low-confidence recommendation, accept or edit workload assumptions, and record the reason for overriding the recommendation.</x:v>
       </x:c>
-      <x:c r="G17" s="26" t="str"/>
+      <x:c r="G17" s="26"/>
     </x:row>
     <x:row r="18" ht="88" customHeight="1">
-      <x:c r="A18" s="20" t="str"/>
+      <x:c r="A18" s="20"/>
       <x:c r="B18" s="20" t="str">
         <x:v>Measurement</x:v>
       </x:c>
@@ -805,12 +805,12 @@
         <x:v>What is one practical metric that would show the agent is useful?</x:v>
       </x:c>
       <x:c r="F18" s="23" t="str">
-        <x:v>Primary metric: CT can produce a first estimate in under three minutes and explain the recommendation plus one alternative tradeoff. Release quality requires all deterministic and governance regression cases to pass and no high-risk or unknown-data case to be marked ready without review.</x:v>
-      </x:c>
-      <x:c r="G18" s="26" t="str"/>
+        <x:v>Primary metric: the decision owner can produce a first estimate in under three minutes and explain the recommendation plus one alternative tradeoff. Release quality requires all deterministic and governance regression cases to pass and no high-risk or unknown-data case to be marked ready without review.</x:v>
+      </x:c>
+      <x:c r="G18" s="26"/>
     </x:row>
     <x:row r="19" ht="88" customHeight="1">
-      <x:c r="A19" s="20" t="str"/>
+      <x:c r="A19" s="20"/>
       <x:c r="B19" s="20" t="str">
         <x:v>Demo</x:v>
       </x:c>
@@ -824,9 +824,9 @@
         <x:v>What will the demo visibly show from input to agent work to human review?</x:v>
       </x:c>
       <x:c r="F19" s="23" t="str">
-        <x:v>The demo opens by asking CT what they are considering building. CT chooses a fast, guided, or safe-example route. The system records Known, Assumed, and Unknown fields; calculates low/expected/high cost; filters ineligible candidates; and shows alternative deltas. Independent Evaluation, Audit, and Governance stages run against a frozen result before the CT Decision Gate becomes available.</x:v>
-      </x:c>
-      <x:c r="G19" s="26" t="str"/>
+        <x:v>The demo opens by asking the product builder what they are considering building. the product builder chooses a fast, guided, or safe-example route. The system records Known, Assumed, and Unknown fields; calculates low/expected/high cost; filters ineligible candidates; and shows alternative deltas. Independent Evaluation, Audit, and Governance stages run against a frozen result before the Human Decision Gate becomes available.</x:v>
+      </x:c>
+      <x:c r="G19" s="26"/>
     </x:row>
     <x:row r="20" ht="88" customHeight="1">
       <x:c r="A20" s="36" t="str">
@@ -847,10 +847,10 @@
       <x:c r="F20" s="34" t="str">
         <x:v>Turn an incomplete AI build idea into an explainable, costed, risk-aware model recommendation that a human can review and use to decide whether and how to proceed.</x:v>
       </x:c>
-      <x:c r="G20" s="34" t="str"/>
+      <x:c r="G20" s="34"/>
     </x:row>
     <x:row r="21" ht="88" customHeight="1">
-      <x:c r="A21" s="20" t="str"/>
+      <x:c r="A21" s="20"/>
       <x:c r="B21" s="20" t="str">
         <x:v>Workflow design</x:v>
       </x:c>
@@ -864,12 +864,12 @@
         <x:v>How does the workflow change when the agent is introduced? List the future process as text steps.</x:v>
       </x:c>
       <x:c r="F21" s="23" t="str">
-        <x:v>1. Ask CT what they are considering building. 2. Route to fast capture, guided questions, or a safe example. 3. After every answer run a completeness check; stop when minimum facts exist or CT selects Estimate now. 4. Freeze a Known/Assumed/Unknown ledger. 5. Load versioned catalog and rules. 6. Calculate real low/expected/high scenarios. 7. Filter hard capability constraints and rank only eligible candidates. 8. Freeze the result. 9. Run independent Evaluation, Audit, and Governance. 10. Return PASS/WARN/REVIEW_REQUIRED/BLOCKED with rule IDs. 11. CT approves, edits, rejects, escalates, or records a permitted override. 12. Export a deterministic decision brief and audit record.</x:v>
-      </x:c>
-      <x:c r="G21" s="26" t="str"/>
+        <x:v>1. Ask the product builder what they are considering building. 2. Route to fast capture, guided questions, or a safe example. 3. After every answer run a completeness check; stop when minimum facts exist or the user selects Estimate now. 4. Freeze a Known/Assumed/Unknown ledger. 5. Load versioned catalog and rules. 6. Calculate real low/expected/high scenarios. 7. Filter hard capability constraints and rank only eligible candidates. 8. Freeze the result. 9. Run independent Evaluation, Audit, and Governance. 10. Return PASS/WARN/REVIEW_REQUIRED/BLOCKED with rule IDs. 11. the product builder approves, edits, rejects, escalates, or records a permitted override. 12. Export a deterministic decision brief and audit record.</x:v>
+      </x:c>
+      <x:c r="G21" s="26"/>
     </x:row>
     <x:row r="22" ht="88" customHeight="1">
-      <x:c r="A22" s="20" t="str"/>
+      <x:c r="A22" s="20"/>
       <x:c r="B22" s="20" t="str">
         <x:v>Agent behavior</x:v>
       </x:c>
@@ -883,12 +883,12 @@
         <x:v>What does the agent observe, reason about, produce, and check before handing work back?</x:v>
       </x:c>
       <x:c r="F22" s="23" t="str">
-        <x:v>The Intake Orchestrator asks only versioned questions and records provenance. The Estimator/Selector is a pure deterministic service and cannot approve. The Evaluator tests the frozen result and cannot mutate it. The Auditor verifies formulas, versions, evidence, and non-mutation. Governance applies absolute rules and cannot recommend or waive findings. CT owns the final judgment. No LLM sits in the recommendation or approval path.</x:v>
-      </x:c>
-      <x:c r="G22" s="26" t="str"/>
+        <x:v>The Intake Orchestrator asks only versioned questions and records provenance. The Estimator/Selector is a pure deterministic service and cannot approve. The Evaluator tests the frozen result and cannot mutate it. The Auditor verifies formulas, versions, evidence, and non-mutation. Governance applies absolute rules and cannot recommend or waive findings. a human owns the final judgment. No LLM sits in the recommendation or approval path.</x:v>
+      </x:c>
+      <x:c r="G22" s="26"/>
     </x:row>
     <x:row r="23" ht="88" customHeight="1">
-      <x:c r="A23" s="20" t="str"/>
+      <x:c r="A23" s="20"/>
       <x:c r="B23" s="20" t="str">
         <x:v>Context</x:v>
       </x:c>
@@ -904,10 +904,10 @@
       <x:c r="F23" s="23" t="str">
         <x:v>User inputs: use case, task types, quality threshold, risk level, data sensitivity, latency, modalities, context, traffic, input/output size, model calls, retrieval, tools, loops, and pinned models. System context: normalized model and price catalog with source date; capability and integration fields; estimation formulas; eligibility and ranking rubric; safety rules; example workload plans; decision-brief format.</x:v>
       </x:c>
-      <x:c r="G23" s="26" t="str"/>
+      <x:c r="G23" s="26"/>
     </x:row>
     <x:row r="24" ht="88" customHeight="1">
-      <x:c r="A24" s="20" t="str"/>
+      <x:c r="A24" s="20"/>
       <x:c r="B24" s="20" t="str">
         <x:v>Tools</x:v>
       </x:c>
@@ -923,10 +923,10 @@
       <x:c r="F24" s="23" t="str">
         <x:v>Implemented prototype tools: prompt-first intake; versioned JSON model catalog; versioned intake and governance rules; deterministic scenario/cost and eligibility engine; fixed evaluation cases; audit invariants; governance dispositions; deterministic decision brief; artifact hub. Purchasing, provisioning, production routing, and deployment authorization remain disabled.</x:v>
       </x:c>
-      <x:c r="G24" s="26" t="str"/>
+      <x:c r="G24" s="26"/>
     </x:row>
     <x:row r="25" ht="88" customHeight="1">
-      <x:c r="A25" s="20" t="str"/>
+      <x:c r="A25" s="20"/>
       <x:c r="B25" s="20" t="str">
         <x:v>Memory</x:v>
       </x:c>
@@ -942,10 +942,10 @@
       <x:c r="F25" s="23" t="str">
         <x:v>Persist the named project, structured workload assumptions, selected catalog version, candidate models, calculations, recommendation, decision status, and override reason. Do not retain secrets, API keys, proprietary source data, protected health information, raw unrelated conversations, or sensitive content copied from a production workload. Users must be able to edit or delete saved plans.</x:v>
       </x:c>
-      <x:c r="G25" s="26" t="str"/>
+      <x:c r="G25" s="26"/>
     </x:row>
     <x:row r="26" ht="88" customHeight="1">
-      <x:c r="A26" s="20" t="str"/>
+      <x:c r="A26" s="20"/>
       <x:c r="B26" s="20" t="str">
         <x:v>Output</x:v>
       </x:c>
@@ -961,10 +961,10 @@
       <x:c r="F26" s="23" t="str">
         <x:v>A one-page decision brief containing: workload summary; assumptions; price-data timestamp; eligible and excluded candidates; low/expected/high cost per request, month, and year; recommended model; alternatives and tradeoffs; largest cost drivers; tuning recommendations; uncertainty and risks; human-review requirement; final decision and override reason.</x:v>
       </x:c>
-      <x:c r="G26" s="26" t="str"/>
+      <x:c r="G26" s="26"/>
     </x:row>
     <x:row r="27" ht="88" customHeight="1">
-      <x:c r="A27" s="20" t="str"/>
+      <x:c r="A27" s="20"/>
       <x:c r="B27" s="20" t="str">
         <x:v>Failure handling</x:v>
       </x:c>
@@ -980,10 +980,10 @@
       <x:c r="F27" s="23" t="str">
         <x:v>Stop and request clarification when required inputs are missing. Mark estimates incomplete when price fields or provider charges are unknown. Do not recommend a model when none meets hard constraints or evidence is insufficient. Require human review for high-risk or regulated workloads, sensitive data, materially consequential decisions, stale catalog data, contradictory rules, or attempted commercial bias. Preserve partial work and explain the blocker.</x:v>
       </x:c>
-      <x:c r="G27" s="26" t="str"/>
+      <x:c r="G27" s="26"/>
     </x:row>
     <x:row r="28" ht="88" customHeight="1">
-      <x:c r="A28" s="20" t="str"/>
+      <x:c r="A28" s="20"/>
       <x:c r="B28" s="20" t="str">
         <x:v>Approval</x:v>
       </x:c>
@@ -999,10 +999,10 @@
       <x:c r="F28" s="23" t="str">
         <x:v>After calculations, eligibility filtering, and the grounded recommendation are displayed—but before the decision is finalized. The user reviews assumptions, sources, exclusions, cost drivers, alternatives, and risk flags; then approves, edits and reruns, selects an alternative with an override reason, rejects the result, or escalates to architecture/governance review.</x:v>
       </x:c>
-      <x:c r="G28" s="26" t="str"/>
+      <x:c r="G28" s="26"/>
     </x:row>
     <x:row r="29" ht="88" customHeight="1">
-      <x:c r="A29" s="20" t="str"/>
+      <x:c r="A29" s="20"/>
       <x:c r="B29" s="20" t="str">
         <x:v>Evaluation</x:v>
       </x:c>
@@ -1018,7 +1018,7 @@
       <x:c r="F29" s="23" t="str">
         <x:v>Use controlled synthetic cases with known cost math and expected rule outcomes. Test a normal text workload, a cheap-model-eligible classification task, a quality-sensitive reasoning task, unsupported modality, excessive agent loops, missing output estimate, stale price data, no eligible model, high-risk medical drafting, and an attempted sponsored-provider bias. Evaluate calculation accuracy, rule consistency, explanation grounding, boundary compliance, and human comprehension.</x:v>
       </x:c>
-      <x:c r="G29" s="26" t="str"/>
+      <x:c r="G29" s="26"/>
     </x:row>
     <x:row r="30" ht="88" customHeight="1">
       <x:c r="A30" s="39" t="str">
@@ -1039,10 +1039,10 @@
       <x:c r="F30" s="37" t="str">
         <x:v>Enter one AI workload plan → identify missing constraints → compare sourced catalog facts across OpenAI, Google, and Anthropic → calculate low/expected/high cost → rank only candidates with shared evidence → explain the recommendation and tuning options → let the human approve or override → display a saved decision brief.</x:v>
       </x:c>
-      <x:c r="G30" s="37" t="str"/>
+      <x:c r="G30" s="37"/>
     </x:row>
     <x:row r="31" ht="88" customHeight="1">
-      <x:c r="A31" s="20" t="str"/>
+      <x:c r="A31" s="20"/>
       <x:c r="B31" s="20" t="str">
         <x:v>Prototype</x:v>
       </x:c>
@@ -1058,10 +1058,10 @@
       <x:c r="F31" s="23" t="str">
         <x:v>The user types a project name and workload description; selects task, risk, latency, and modality; enters traffic, input/output, calls, retrieval, tools, and loop assumptions; pins or accepts suggested models; clicks Calculate and Compare; reviews cost cards, exclusions, recommendation, and tuning; changes an assumption; reruns; then approves or overrides the decision.</x:v>
       </x:c>
-      <x:c r="G31" s="26" t="str"/>
+      <x:c r="G31" s="26"/>
     </x:row>
     <x:row r="32" ht="88" customHeight="1">
-      <x:c r="A32" s="20" t="str"/>
+      <x:c r="A32" s="20"/>
       <x:c r="B32" s="20" t="str">
         <x:v>Data</x:v>
       </x:c>
@@ -1077,10 +1077,10 @@
       <x:c r="F32" s="23" t="str">
         <x:v>Implemented demo-safe inputs: a versioned catalog containing dated published facts for three OpenAI, two Google Gemini, and three Anthropic Claude models; versioned intake, eligibility, and governance rules; deterministic cost scenarios; ten fictional evaluation cases; and a synthetic RAG customer-support workload used in the demo. No secret, customer, employer, medical, or proprietary data is required.</x:v>
       </x:c>
-      <x:c r="G32" s="26" t="str"/>
+      <x:c r="G32" s="26"/>
     </x:row>
     <x:row r="33" ht="88" customHeight="1">
-      <x:c r="A33" s="20" t="str"/>
+      <x:c r="A33" s="20"/>
       <x:c r="B33" s="20" t="str">
         <x:v>Evaluation</x:v>
       </x:c>
@@ -1096,10 +1096,10 @@
       <x:c r="F33" s="23" t="str">
         <x:v>1. Happy path: text RAG support agent with complete assumptions and multiple eligible models. 2. Simple classification: economical model should pass and outrank premium model. 3. Missing output estimate: agent must ask for clarification and not create false precision. 4. Unsupported image modality: text-only model must be excluded. 5. Excessive loops: cost warning and loop-cap recommendation. 6. High-risk medical draft: mandatory human review and no autonomous approval. 7. Stale price catalog: visible warning and blocked final recommendation. 8. No eligible model: stop and escalate rather than force a choice.</x:v>
       </x:c>
-      <x:c r="G33" s="26" t="str"/>
+      <x:c r="G33" s="26"/>
     </x:row>
     <x:row r="34" ht="88" customHeight="1">
-      <x:c r="A34" s="20" t="str"/>
+      <x:c r="A34" s="20"/>
       <x:c r="B34" s="20" t="str">
         <x:v>Evaluation</x:v>
       </x:c>
@@ -1113,12 +1113,12 @@
         <x:v>What happened when you tested the agent? Where did it pass, fail, or need a human?</x:v>
       </x:c>
       <x:c r="F34" s="46" t="str">
-        <x:v>Observed governed-alpha results on August 8, 2026: 10 automated tests passed and 0 failed. Evidence covers same-input determinism, ordered low/expected/high scenarios, high-risk human review, unknown-data fail-closed behavior, unsupported modality blocking, stale-pricing blocking, visible assumption warnings, agent-loop warning/block thresholds, candidate-order invariance, and rendered-app smoke coverage. The production build completed all five stages without an AI credential.</x:v>
-      </x:c>
-      <x:c r="G34" s="26" t="str"/>
+        <x:v>Observed governed-alpha results on August 8, 2026: 11 automated tests passed and 0 failed. Evidence covers same-input determinism, ordered low/expected/high scenarios, high-risk human review, unknown-data fail-closed behavior, unsupported modality blocking, stale-pricing blocking, visible assumption warnings, agent-loop warning/block thresholds, candidate-order invariance, and rendered-app smoke coverage. The production build completed all five stages without an AI credential.</x:v>
+      </x:c>
+      <x:c r="G34" s="26"/>
     </x:row>
     <x:row r="35" ht="88" customHeight="1">
-      <x:c r="A35" s="20" t="str"/>
+      <x:c r="A35" s="20"/>
       <x:c r="B35" s="20" t="str">
         <x:v>Iteration</x:v>
       </x:c>
@@ -1132,12 +1132,12 @@
         <x:v>What did you change after testing, and why?</x:v>
       </x:c>
       <x:c r="F35" s="46" t="str">
-        <x:v>The live generative decision-brief route was removed so no LLM can influence recommendation or approval. The all-at-once form now begins with fast, guided, and safe-example routes. Field provenance, versioned rules/catalog, real scenario ranges, independent Evaluation/Audit/Governance, fail-closed dispositions, and the CT Decision Gate were added. GitHub Pages became an artifact hub instead of a duplicated calculator so decision logic cannot drift.</x:v>
-      </x:c>
-      <x:c r="G35" s="26" t="str"/>
+        <x:v>The live generative decision-brief route was removed so no LLM can influence recommendation or approval. The all-at-once form now begins with fast, guided, and safe-example routes. Field provenance, versioned rules/catalog, real scenario ranges, independent Evaluation/Audit/Governance, fail-closed dispositions, and the Human Decision Gate were added. GitHub Pages became an artifact hub instead of a duplicated calculator so decision logic cannot drift.</x:v>
+      </x:c>
+      <x:c r="G35" s="26"/>
     </x:row>
     <x:row r="36" ht="88" customHeight="1">
-      <x:c r="A36" s="20" t="str"/>
+      <x:c r="A36" s="20"/>
       <x:c r="B36" s="20" t="str">
         <x:v>Constraints</x:v>
       </x:c>
@@ -1151,12 +1151,12 @@
         <x:v>What does the prototype not do yet? Be honest and specific.</x:v>
       </x:c>
       <x:c r="F36" s="23" t="str">
-        <x:v>The alpha compares sourced catalog facts across three providers, but only the evaluated baseline can enter the recommendation ranking. It will not infer universal model quality, purchase or provision access, automatically route production traffic, ingest secrets or protected data, monitor real production spend, approve regulated deployments, cover every provider fee, guarantee future pricing, or implement monetization and stored-value credits. The tool is authoritative for its versioned inputs, sourced facts, deterministic calculations, and recorded policy disposition; CT remains the decision owner.</x:v>
-      </x:c>
-      <x:c r="G36" s="26" t="str"/>
+        <x:v>The alpha compares sourced catalog facts across three providers, but only the evaluated baseline can enter the recommendation ranking. It will not infer universal model quality, purchase or provision access, automatically route production traffic, ingest secrets or protected data, monitor real production spend, approve regulated deployments, cover every provider fee, guarantee future pricing, or implement monetization and stored-value credits. The tool is authoritative for its versioned inputs, sourced facts, deterministic calculations, and recorded policy disposition; the product builder remains the decision owner.</x:v>
+      </x:c>
+      <x:c r="G36" s="26"/>
     </x:row>
     <x:row r="37" ht="88" customHeight="1">
-      <x:c r="A37" s="20" t="str"/>
+      <x:c r="A37" s="20"/>
       <x:c r="B37" s="20" t="str">
         <x:v>Demo</x:v>
       </x:c>
@@ -1170,9 +1170,9 @@
         <x:v>Describe what the working prototype shows. A reviewer should understand the demo loop from this text.</x:v>
       </x:c>
       <x:c r="F37" s="46" t="str">
-        <x:v>The working governed alpha asks CT what they are considering building, offers fast/guided/safe-example routes, and provides an Estimate now escape hatch. A workload-freeze panel captures task, risk, data, regulation, modality, traffic, tokens, cache, calls, and context while showing provenance. The deterministic result displays low/expected/high cost, the least expensive rule-eligible model, alternative cost deltas, and exclusions. Evaluation, Audit, and Governance show their statuses and rule findings before the CT Decision Gate. The full app is on OpenAI Sites; GitHub Pages is the artifact hub.</x:v>
-      </x:c>
-      <x:c r="G37" s="26" t="str"/>
+        <x:v>The working governed alpha asks the product builder what they are considering building, offers fast/guided/safe-example routes, and provides an Estimate now escape hatch. A workload-freeze panel captures task, risk, data, regulation, modality, traffic, tokens, cache, calls, and context while showing provenance. The deterministic result displays low/expected/high cost, the least expensive rule-eligible model, alternative cost deltas, and exclusions. Evaluation, Audit, and Governance show their statuses and rule findings before the Human Decision Gate. The full app is on OpenAI Sites; GitHub Pages is the artifact hub.</x:v>
+      </x:c>
+      <x:c r="G37" s="26"/>
     </x:row>
     <x:row r="38" ht="88" customHeight="1">
       <x:c r="A38" s="42" t="str">
@@ -1191,12 +1191,12 @@
         <x:v>Would you pilot this? What still needs to be true before launch?</x:v>
       </x:c>
       <x:c r="F38" s="40" t="str">
-        <x:v>Go for a CT-only alpha using synthetic or non-sensitive planning assumptions. The deterministic and governance suite passes 10 of 10. No-go for medical-billing production decisions, purchasing, automated routing, or protected content. Before external pilots: complete CT usability sessions, persist an append-only decision record with deletion controls, add accessibility regression coverage, and validate provider catalogs and task-specific quality evidence.</x:v>
-      </x:c>
-      <x:c r="G38" s="40" t="str"/>
+        <x:v>Go for a small alpha using synthetic or non-sensitive planning assumptions. The deterministic and governance suite passes 10 of 10. No-go for medical-billing production decisions, purchasing, automated routing, or protected content. Before external pilots: complete the product builder usability sessions, persist an append-only decision record with deletion controls, add accessibility regression coverage, and validate provider catalogs and task-specific quality evidence.</x:v>
+      </x:c>
+      <x:c r="G38" s="40"/>
     </x:row>
     <x:row r="39" ht="88" customHeight="1">
-      <x:c r="A39" s="20" t="str"/>
+      <x:c r="A39" s="20"/>
       <x:c r="B39" s="20" t="str">
         <x:v>Risk</x:v>
       </x:c>
@@ -1212,10 +1212,10 @@
       <x:c r="F39" s="23" t="str">
         <x:v>Risks include stale or incorrect prices; fabricated model capabilities; misleading precision; poor model-fit recommendations; users entering secrets, proprietary data, or protected information; commercial bias; overreliance on generated explanations; and use of the result as deployment approval. Controls include minimal data collection, source timestamps, structured calculations, eligibility rules, visible uncertainty, human approval, audit history, deletion, and commercial disclosure.</x:v>
       </x:c>
-      <x:c r="G39" s="26" t="str"/>
+      <x:c r="G39" s="26"/>
     </x:row>
     <x:row r="40" ht="88" customHeight="1">
-      <x:c r="A40" s="20" t="str"/>
+      <x:c r="A40" s="20"/>
       <x:c r="B40" s="20" t="str">
         <x:v>Operations</x:v>
       </x:c>
@@ -1229,12 +1229,12 @@
         <x:v>Who reviews agent output, handles escalations, and owns final decisions?</x:v>
       </x:c>
       <x:c r="F40" s="23" t="str">
-        <x:v>For the alpha, CT owns workload assumptions and the final decision. Estimation, Evaluation, Audit, and Governance have separate hard-bordered contracts and cannot waive one another's findings. Architecture, security, privacy, procurement, or medical-domain specialists own escalations in their areas. The system does not own purchase, deployment, risk acceptance, budget approval, or regulated-use authorization.</x:v>
-      </x:c>
-      <x:c r="G40" s="26" t="str"/>
+        <x:v>For the alpha, a human owns workload assumptions and the final decision. Estimation, Evaluation, Audit, and Governance have separate hard-bordered contracts and cannot waive one another's findings. Architecture, security, privacy, procurement, or medical-domain specialists own escalations in their areas. The system does not own purchase, deployment, risk acceptance, budget approval, or regulated-use authorization.</x:v>
+      </x:c>
+      <x:c r="G40" s="26"/>
     </x:row>
     <x:row r="41" ht="88" customHeight="1">
-      <x:c r="A41" s="20" t="str"/>
+      <x:c r="A41" s="20"/>
       <x:c r="B41" s="20" t="str">
         <x:v>Monitoring</x:v>
       </x:c>
@@ -1250,10 +1250,10 @@
       <x:c r="F41" s="23" t="str">
         <x:v>Monitor catalog freshness and failed refreshes; estimate versus actual usage and cost; calculation errors; recommendation and override rates; no-eligible-model frequency; stale-data warnings; explanation-to-structured-result consistency; user-reported incorrect capability claims; high-risk escalations; sensitive-data attempts; latency; task completion; and whether recommended models continue to pass representative evaluations.</x:v>
       </x:c>
-      <x:c r="G41" s="26" t="str"/>
+      <x:c r="G41" s="26"/>
     </x:row>
     <x:row r="42" ht="88" customHeight="1">
-      <x:c r="A42" s="20" t="str"/>
+      <x:c r="A42" s="20"/>
       <x:c r="B42" s="20" t="str">
         <x:v>Feedback</x:v>
       </x:c>
@@ -1269,10 +1269,10 @@
       <x:c r="F42" s="23" t="str">
         <x:v>After each decision brief, ask whether the recommendation was understandable, useful, trusted, and acted on; capture the reason for overrides; interview pilot users about missing criteria and research time; compare estimates with actual usage when available; review failure and escalation cases weekly; and prioritize changes by decision harm, frequency, user impact, and evidence—not by feature requests alone.</x:v>
       </x:c>
-      <x:c r="G42" s="26" t="str"/>
+      <x:c r="G42" s="26"/>
     </x:row>
     <x:row r="43" ht="88" customHeight="1">
-      <x:c r="A43" s="20" t="str"/>
+      <x:c r="A43" s="20"/>
       <x:c r="B43" s="20" t="str">
         <x:v>Rollout</x:v>
       </x:c>
@@ -1286,12 +1286,12 @@
         <x:v>What is the smallest safe launch or pilot path?</x:v>
       </x:c>
       <x:c r="F43" s="23" t="str">
-        <x:v>Begin with CT and synthetic or non-sensitive workloads using the three-provider catalog. Run three real planning sessions plus high-risk, stale-catalog, and unsupported-modality failure demos. Next invite three to five product builders with fictional or sanitized plans. Connect Google Gemini and Anthropic Claude to shared live evaluation only after provider-key, budget, synthetic-case, adapter, source, freshness, and ranking-bias tests pass.</x:v>
-      </x:c>
-      <x:c r="G43" s="26" t="str"/>
+        <x:v>Begin with the product builder and synthetic or non-sensitive workloads using the three-provider catalog. Run three real planning sessions plus high-risk, stale-catalog, and unsupported-modality failure demos. Next invite three to five product builders with fictional or sanitized plans. Connect Google Gemini and Anthropic Claude to shared live evaluation only after provider-key, budget, synthetic-case, adapter, source, freshness, and ranking-bias tests pass.</x:v>
+      </x:c>
+      <x:c r="G43" s="26"/>
     </x:row>
     <x:row r="44" ht="88" customHeight="1">
-      <x:c r="A44" s="20" t="str"/>
+      <x:c r="A44" s="20"/>
       <x:c r="B44" s="20" t="str">
         <x:v>Communication</x:v>
       </x:c>
@@ -1305,9 +1305,9 @@
         <x:v>How will your video cover intro, problem, discovery, solution demo, eval rigor, impact, and launch plan?</x:v>
       </x:c>
       <x:c r="F44" s="23" t="str">
-        <x:v>0:00–0:25 Explain fragmented model choice and bad defaults. 0:25–0:45 Introduce AI Build Crew and CT. 0:45–1:15 Show prompt-first routing and Known/Assumed/Unknown. 1:15–1:45 Show three-provider catalog facts, scenarios, rule eligibility, and evidence-gated ranking. 1:45–2:10 Show independent Evaluation, Audit, Governance, and CT ownership. 2:10–2:30 State 10/10 evidence, limitations, and shared live evaluation as the next step.</x:v>
-      </x:c>
-      <x:c r="G44" s="26" t="str"/>
+        <x:v>0:00–0:25 Explain fragmented model choice and bad defaults. 0:25–0:45 Introduce AI Build Crew and the product builder. 0:45–1:15 Show prompt-first routing and Known/Assumed/Unknown. 1:15–1:45 Show three-provider catalog facts, scenarios, rule eligibility, and evidence-gated ranking. 1:45–2:10 Show independent Evaluation, Audit, Governance, and the product builder ownership. 2:10–2:30 State 11/11 evidence, limitations, and shared live evaluation as the next step.</x:v>
+      </x:c>
+      <x:c r="G44" s="26"/>
     </x:row>
     <x:row r="45" ht="88" customHeight="1">
       <x:c r="A45" s="45" t="str">
@@ -1326,12 +1326,12 @@
         <x:v>Is every grading-critical decision written directly in this sheet with no required link-outs?</x:v>
       </x:c>
       <x:c r="F45" s="47" t="str">
-        <x:v>YES. Discovery, design, implemented scope, deterministic architecture, specialist boundaries, absolute rules, observed 10/10 evaluation evidence, iteration, working-demo behavior, limitations, readiness, and rollout are written directly in this sheet.</x:v>
-      </x:c>
-      <x:c r="G45" s="43" t="str"/>
+        <x:v>YES. Discovery, design, implemented scope, deterministic architecture, specialist boundaries, absolute rules, observed 11/11 evaluation evidence, iteration, working-demo behavior, limitations, readiness, and rollout are written directly in this sheet.</x:v>
+      </x:c>
+      <x:c r="G45" s="43"/>
     </x:row>
     <x:row r="46" ht="88" customHeight="1">
-      <x:c r="A46" s="20" t="str"/>
+      <x:c r="A46" s="20"/>
       <x:c r="B46" s="20" t="str">
         <x:v>Submission</x:v>
       </x:c>
@@ -1345,12 +1345,12 @@
         <x:v>Can a reviewer understand the working prototype loop from the PRD and video?</x:v>
       </x:c>
       <x:c r="F46" s="46" t="str">
-        <x:v>YES FOR THE PRD AND SCRIPT. The prompt-first routes, provenance ledger, scenario calculation, eligibility filtering, recommendation/alternatives, independent checks, CT Decision Gate, and known omissions are described directly above. The final recording should follow the supplied 2–3 minute script.</x:v>
-      </x:c>
-      <x:c r="G46" s="26" t="str"/>
+        <x:v>YES FOR THE PRD AND SCRIPT. The prompt-first routes, provenance ledger, scenario calculation, eligibility filtering, recommendation/alternatives, independent checks, Human Decision Gate, and known omissions are described directly above. The final recording should follow the supplied 2–3 minute script.</x:v>
+      </x:c>
+      <x:c r="G46" s="26"/>
     </x:row>
     <x:row r="47" ht="88" customHeight="1">
-      <x:c r="A47" s="21" t="str"/>
+      <x:c r="A47" s="21"/>
       <x:c r="B47" s="21" t="str">
         <x:v>Submission</x:v>
       </x:c>
@@ -1366,7 +1366,7 @@
       <x:c r="F47" s="48" t="str">
         <x:v>READY TO RECORD. A timed 2:30 script and operator checklist are complete. Before submission, record it, verify runtime, confirm the high-risk review state is visible, and check that the narration matches the PRD, evaluation, limitations, three-provider catalog, and shared-evaluation next step.</x:v>
       </x:c>
-      <x:c r="G47" s="27" t="str"/>
+      <x:c r="G47" s="27"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>